<commit_message>
Add categories for the WD 4 and WD 5 Fachbereiche (#243)
FI (Haushalt und Finanzen) and WI (Wirtschaft, Energie, Umwelt), plus the
mapping from a Fachbereich or Aktenzeichen to its category, which the Word
reader for the reviewers' template needs because that template has no
category column. The collection templates are regenerated so their help text
lists the new categories.
</commit_message>
<xml_diff>
--- a/evaluation/vorlagen/SENTRA-Testfaelle-Erfassung.xlsx
+++ b/evaluation/vorlagen/SENTRA-Testfaelle-Erfassung.xlsx
@@ -191,7 +191,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte.</t>
+        <t>Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte; FI = Haushalt und Finanzen; WI = Wirtschaft, Energie, Umwelt.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -4202,8 +4202,8 @@
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="2">
-    <dataValidation sqref="A2:A301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Kategorie" error="Bitte einen Wert aus der Liste wählen." promptTitle="Kategorie" prompt="Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte." type="list">
-      <formula1>"GO,GV,AR"</formula1>
+    <dataValidation sqref="A2:A301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Kategorie" error="Bitte einen Wert aus der Liste wählen." promptTitle="Kategorie" prompt="Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte; FI = Haushalt und Finanzen; WI = Wirtschaft, Energie, Umwelt." type="list">
+      <formula1>"GO,GV,AR,FI,WI"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Grenzfall?" error="Bitte einen Wert aus der Liste wählen." promptTitle="Grenzfall?" prompt="„ja“, wenn der Bestand die Frage bewusst nicht abdeckt und SENTRA die Antwort verweigern soll. Grenzfälle werden immer manuell geprüft und nie automatisch herausgefiltert — sie sind die riskanteste Kategorie: ein System, das etwas erfindet, ist schlimmer als eines, das nichts findet." type="list">
       <formula1>"nein,ja"</formula1>
@@ -4289,7 +4289,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Kategorie *</t>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte.</t>
+          <t>Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte; FI = Haushalt und Finanzen; WI = Wirtschaft, Energie, Umwelt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add categories for the WD 4 and WD 5 Fachbereiche (#243) (#246)
FI (Haushalt und Finanzen) and WI (Wirtschaft, Energie, Umwelt), plus the
mapping from a Fachbereich or Aktenzeichen to its category, which the Word
reader for the reviewers' template needs because that template has no
category column. The collection templates are regenerated so their help text
lists the new categories.
</commit_message>
<xml_diff>
--- a/evaluation/vorlagen/SENTRA-Testfaelle-Erfassung.xlsx
+++ b/evaluation/vorlagen/SENTRA-Testfaelle-Erfassung.xlsx
@@ -191,7 +191,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte.</t>
+        <t>Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte; FI = Haushalt und Finanzen; WI = Wirtschaft, Energie, Umwelt.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -4202,8 +4202,8 @@
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="2">
-    <dataValidation sqref="A2:A301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Kategorie" error="Bitte einen Wert aus der Liste wählen." promptTitle="Kategorie" prompt="Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte." type="list">
-      <formula1>"GO,GV,AR"</formula1>
+    <dataValidation sqref="A2:A301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Kategorie" error="Bitte einen Wert aus der Liste wählen." promptTitle="Kategorie" prompt="Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte; FI = Haushalt und Finanzen; WI = Wirtschaft, Energie, Umwelt." type="list">
+      <formula1>"GO,GV,AR,FI,WI"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J301" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Grenzfall?" error="Bitte einen Wert aus der Liste wählen." promptTitle="Grenzfall?" prompt="„ja“, wenn der Bestand die Frage bewusst nicht abdeckt und SENTRA die Antwort verweigern soll. Grenzfälle werden immer manuell geprüft und nie automatisch herausgefiltert — sie sind die riskanteste Kategorie: ein System, das etwas erfindet, ist schlimmer als eines, das nichts findet." type="list">
       <formula1>"nein,ja"</formula1>
@@ -4289,7 +4289,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Kategorie *</t>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte.</t>
+          <t>Grobe Einordnung der Frage. Bestimmt die Test-ID. GO = Geschäftsordnung; GV = Gesetzgebungsverfahren; AR = Abgeordnetenrechte; FI = Haushalt und Finanzen; WI = Wirtschaft, Energie, Umwelt.</t>
         </is>
       </c>
     </row>

</xml_diff>